<commit_message>
docs: architecture PNG diagrams + web/mobile parity
</commit_message>
<xml_diff>
--- a/data/DATA_WAR_TIKET_KONSER.xlsx
+++ b/data/DATA_WAR_TIKET_KONSER.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="26940" windowHeight="13900" tabRatio="600" firstSheet="10" activeTab="18" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="00_Panduan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="01_Ownership" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="02_Data_Dictionary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="03_venues" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="04_events" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="05_seat_categories" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="06_seat_map" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="07_seat_inventory" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="08_holds" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="09_tickets" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="10_transactions" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="11_payment_attempts" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="12_notification_jobs" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="13_delivery_logs" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="14_users_sample" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="15_redis_keys" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="18_seed_checklist" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="16_enums_status" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="17_relasi_ER" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Panduan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Ownership" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Data_Dictionary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_venues" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_events" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_seat_categories" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_seat_map" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_seat_inventory" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_holds" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_tickets" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_transactions" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_payment_attempts" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_notification_jobs" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_delivery_logs" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_users_sample" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_redis_keys" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_seed_checklist" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_enums_status" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_relasi_ER" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -33,7 +33,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -5193,7 +5195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
     <col width="11.33203125" customWidth="1" min="1" max="1"/>
@@ -5627,6 +5629,671 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>VEN012</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>JAMSIL-MAIN</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Jamsil Olympic Main Stadium</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Seoul</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>25 Olympic-ro, Songpa-gu, Seoul</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>420</v>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>VEN013</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>KINTEX-HALL</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>KINTEX Exhibition Center Hall A</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Goyang</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>217-60 Kintex-ro, Ilsanseo-gu, Goyang</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>380</v>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>VEN014</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>GOYANG-STAD</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Goyang Stadium</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Goyang</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>890 Jungang-ro, Ilsandong-gu, Goyang</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>480</v>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>VEN015</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>KAOHSIUNG-ARENA</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Kaohsiung Arena</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Kaohsiung</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>No. 111, Zhongshan 1st Rd, Qianjin District, Kaohsiung</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>340</v>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>VEN016</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>TOKYO-DOME-C</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Tokyo Dome City Hall</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Tokyo</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>1-3-61 Koraku, Bunkyo City, Tokyo</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>310</v>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>VEN017</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>DAEGU-EXCO</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>EXCO Daegu Convention Hall</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Daegu</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>10 Exco-ro, Buk-gu, Daegu</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>290</v>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>VEN018</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>JAKARTA-JIS</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Jakarta International Stadium</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Jalan Laksamana Yos Sudarso, Tanjung Priok, Jakarta</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>VEN019</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>SINGAPORE-NS</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Singapore National Stadium</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>1 Stadium Drive, Singapore</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>450</v>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>VEN020</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>OLYMPIC-GYM</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Olympic Gymnastics Arena</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Seoul</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>424 Olympic-ro, Songpa-gu, Seoul</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>330</v>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>VEN021</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>SNU-STAD</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Seoul Olympic Stadium</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Seoul</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>25 Olympic-ro, Songpa-gu, Seoul</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>500</v>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>VEN022</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>INSPIRE-HALL</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Inspire Arena Hall B</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Incheon</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>127 Gonghangmunhwa-ro, Jung-gu, Incheon</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>370</v>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>VEN023</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>JAMSIL-INDOOR2</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Jamsil Indoor Stadium Hall 2</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Seoul</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>25 Olympic-ro, Songpa-gu, Seoul</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>340</v>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>VEN024</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>BEXCO-AUD2</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>BEXCO Auditorium 2</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Busan</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>55 APEC-ro, Haeundae-gu, Busan</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>310</v>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>VEN025</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>KSPO-DOME2</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>KSPO DOME Hall Annex</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Seoul</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Olympic-ro 424, Songpa-gu, Seoul</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>VEN026</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>TOKYO-FORUM</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Tokyo International Forum Hall A</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Tokyo</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>3-5-1 Marunouchi, Chiyoda City, Tokyo</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>340</v>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>VEN027</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>IMPACT-HALL5</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>IMPACT Exhibition Hall 5</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Bangkok Metro</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Popular Rd, Ban Mai, Pak Kret, Nonthaburi, Thailand</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>300</v>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>VEN028</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>ICE-BSD</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Indonesia Convention Exhibition (ICE) BSD</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>Tangerang</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>BSD City, Tangerang Selatan, Banten</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>VEN029</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>OLYMPIC-HALL2</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Olympic Hall Side A</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Seoul</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>424 Olympic-ro, Songpa-gu, Seoul</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>310</v>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>VEN030</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>CRYPTO-COM</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Crypto.com Arena</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>1111 S Figueroa St, Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>370</v>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5638,7 +6305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
     <col width="11.1640625" customWidth="1" min="1" max="1"/>
@@ -6155,6 +6822,690 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>EVT012</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>IU-SEOUL</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>IU (아이유)</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>VEN012</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>46302.79166666666</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>46262.41666666666</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>46301.91666666666</v>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>EVT013</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>NJ-GOYANG</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>NewJeans (뉴진스)</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>VEN013</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>46317.79166666666</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>46282.41666666666</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>46316.91666666666</v>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>EVT014</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>SVT-ENC</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>SEVENTEEN (세븐틴) ENCORE</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>VEN014</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>46332.79166666666</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>46282.41666666666</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>46331.91666666666</v>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>EVT015</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>TWICE-KHH</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>TWICE (트와이스)</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>VEN015</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>46347.79166666666</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>46302.41666666666</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>46346.91666666666</v>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>EVT016</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>LSF-TKY</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>LE SSERAFIM (르세라핌)</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>VEN016</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>46357.79166666666</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>46317.41666666666</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>46356.91666666666</v>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>EVT017</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>ITZY-DGU</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>ITZY (있지)</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>VEN017</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>46367.79166666666</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>46337.41666666666</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>46366.91666666666</v>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>EVT018</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>GIDLE-JKT</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>(G)I-DLE ((여자)아이들)</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>VEN018</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>46377.79166666666</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>46322.41666666666</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>46376.91666666666</v>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>EVT019</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>ENH-SG</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>ENHYPEN (엔하이픈)</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>VEN019</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>46392.79166666666</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>46342.41666666666</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>46391.91666666666</v>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>EVT020</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>IVE-SEOUL</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>IVE (아이브)</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>VEN020</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>46407.79166666666</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>46362.41666666666</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>46406.91666666666</v>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>EVT021</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>BTS-SEOUL</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>BTS (방탄소년단)</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>VEN021</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>46417.79166666666</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>46367.41666666666</v>
+      </c>
+      <c r="G22" s="9" t="n">
+        <v>46416.91666666666</v>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>EVT022</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>TXT-ICN</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>TOMORROW X TOGETHER (투모로우바이투게더)</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>VEN022</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>46427.79166666666</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>46387.41666666666</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>46426.91666666666</v>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>EVT023</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>RIIZE-SEOUL</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>RIIZE (라이즈)</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>VEN023</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>46437.79166666666</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>46402.41666666666</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>46436.91666666666</v>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>EVT024</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>BOYNEXTDOOR-BSN</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>BOYNEXTDOOR (보이넥스트도어)</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>VEN024</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>46447.79166666666</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>46417.41666666666</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>46446.91666666666</v>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>EVT025</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>ZB1-SEOUL</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>ZEROBASEONE (제로베이스원)</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>VEN025</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>46457.79166666666</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>46412.41666666666</v>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>46456.91666666666</v>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>EVT026</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>KISS-OF-LIFE-TKY</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>KISS OF LIFE (키스오브라이프)</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>VEN026</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>46467.79166666666</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>46427.41666666666</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>46466.91666666666</v>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>EVT027</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>NMIXX-BKK</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>NMIXX (엔믹스)</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>VEN027</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>46477.79166666666</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>46442.41666666666</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>46476.91666666666</v>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>EVT028</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>BABYMONSTER-JKT</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>BABYMONSTER (베이비몬스터)</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>VEN028</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>46487.79166666666</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>46437.41666666666</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>46486.91666666666</v>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>EVT029</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>ILLIT-SEOUL</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>ILLIT (아일릿)</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>VEN029</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>46497.79166666666</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>46467.41666666666</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>46496.91666666666</v>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>EVT030</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>KATSEYE-LA</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>KATSEYE</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>VEN030</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>46507.79166666666</v>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>46462.41666666666</v>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>46506.91666666666</v>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6166,7 +7517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G123"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" customWidth="1" min="1" max="1"/>
@@ -7629,6 +8980,2613 @@
         <v>70</v>
       </c>
       <c r="G44" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>CAT044</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>EVT012</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>4800000</v>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>CAT045</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>EVT012</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>CAT046</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>EVT012</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>Gold Lower</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>2800000</v>
+      </c>
+      <c r="F47" s="9" t="n">
+        <v>140</v>
+      </c>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>CAT047</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>EVT012</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>Silver Upper</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="n">
+        <v>1900000</v>
+      </c>
+      <c r="F48" s="9" t="n">
+        <v>140</v>
+      </c>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>CAT048</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>EVT013</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>SCVIP</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>Soundcheck VIP</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="n">
+        <v>5200000</v>
+      </c>
+      <c r="F49" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>CAT049</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>EVT013</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="n">
+        <v>4100000</v>
+      </c>
+      <c r="F50" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>CAT050</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>EVT013</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="F51" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>CAT051</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>EVT013</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>ORANGE</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>Orange Bowl</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>CAT052</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>EVT013</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>NAVY</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>Navy Upper</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="n">
+        <v>1700000</v>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>CAT053</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>EVT014</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="F54" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>CAT054</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>EVT014</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="n">
+        <v>3300000</v>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>140</v>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>CAT055</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>EVT014</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>Gold Lower</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="n">
+        <v>2600000</v>
+      </c>
+      <c r="F56" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="G56" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>CAT056</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>EVT014</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>Silver Upper</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="F57" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="G57" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>CAT057</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>EVT015</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>VVIP</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>VVIP Front</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="n">
+        <v>4600000</v>
+      </c>
+      <c r="F58" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="G58" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>CAT058</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>EVT015</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E59" s="9" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="F59" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G59" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>CAT059</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>EVT015</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>A Reserved</t>
+        </is>
+      </c>
+      <c r="E60" s="9" t="n">
+        <v>2700000</v>
+      </c>
+      <c r="F60" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="G60" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>CAT060</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="inlineStr">
+        <is>
+          <t>EVT015</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D61" s="9" t="inlineStr">
+        <is>
+          <t>B Reserved</t>
+        </is>
+      </c>
+      <c r="E61" s="9" t="n">
+        <v>1900000</v>
+      </c>
+      <c r="F61" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="G61" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>CAT061</t>
+        </is>
+      </c>
+      <c r="B62" s="9" t="inlineStr">
+        <is>
+          <t>EVT016</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D62" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E62" s="9" t="n">
+        <v>4300000</v>
+      </c>
+      <c r="F62" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="G62" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t>CAT062</t>
+        </is>
+      </c>
+      <c r="B63" s="9" t="inlineStr">
+        <is>
+          <t>EVT016</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D63" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E63" s="9" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="F63" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G63" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>CAT063</t>
+        </is>
+      </c>
+      <c r="B64" s="9" t="inlineStr">
+        <is>
+          <t>EVT016</t>
+        </is>
+      </c>
+      <c r="C64" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D64" s="9" t="inlineStr">
+        <is>
+          <t>Gold Seat</t>
+        </is>
+      </c>
+      <c r="E64" s="9" t="n">
+        <v>2300000</v>
+      </c>
+      <c r="F64" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G64" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="9" t="inlineStr">
+        <is>
+          <t>CAT064</t>
+        </is>
+      </c>
+      <c r="B65" s="9" t="inlineStr">
+        <is>
+          <t>EVT016</t>
+        </is>
+      </c>
+      <c r="C65" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="inlineStr">
+        <is>
+          <t>Silver Seat</t>
+        </is>
+      </c>
+      <c r="E65" s="9" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="F65" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="G65" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="9" t="inlineStr">
+        <is>
+          <t>CAT065</t>
+        </is>
+      </c>
+      <c r="B66" s="9" t="inlineStr">
+        <is>
+          <t>EVT017</t>
+        </is>
+      </c>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E66" s="9" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="F66" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="G66" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="inlineStr">
+        <is>
+          <t>CAT066</t>
+        </is>
+      </c>
+      <c r="B67" s="9" t="inlineStr">
+        <is>
+          <t>EVT017</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E67" s="9" t="n">
+        <v>2700000</v>
+      </c>
+      <c r="F67" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="G67" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="9" t="inlineStr">
+        <is>
+          <t>CAT067</t>
+        </is>
+      </c>
+      <c r="B68" s="9" t="inlineStr">
+        <is>
+          <t>EVT017</t>
+        </is>
+      </c>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D68" s="9" t="inlineStr">
+        <is>
+          <t>Gold Lower</t>
+        </is>
+      </c>
+      <c r="E68" s="9" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="F68" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G68" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="inlineStr">
+        <is>
+          <t>CAT068</t>
+        </is>
+      </c>
+      <c r="B69" s="9" t="inlineStr">
+        <is>
+          <t>EVT017</t>
+        </is>
+      </c>
+      <c r="C69" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="inlineStr">
+        <is>
+          <t>Silver Upper</t>
+        </is>
+      </c>
+      <c r="E69" s="9" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="F69" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="G69" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>CAT069</t>
+        </is>
+      </c>
+      <c r="B70" s="9" t="inlineStr">
+        <is>
+          <t>EVT018</t>
+        </is>
+      </c>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E70" s="9" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="F70" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G70" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="inlineStr">
+        <is>
+          <t>CAT070</t>
+        </is>
+      </c>
+      <c r="B71" s="9" t="inlineStr">
+        <is>
+          <t>EVT018</t>
+        </is>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>Festival Standing</t>
+        </is>
+      </c>
+      <c r="E71" s="9" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="F71" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="G71" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="9" t="inlineStr">
+        <is>
+          <t>CAT071</t>
+        </is>
+      </c>
+      <c r="B72" s="9" t="inlineStr">
+        <is>
+          <t>EVT018</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>Gold Tribune</t>
+        </is>
+      </c>
+      <c r="E72" s="9" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="F72" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="G72" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="inlineStr">
+        <is>
+          <t>CAT072</t>
+        </is>
+      </c>
+      <c r="B73" s="9" t="inlineStr">
+        <is>
+          <t>EVT018</t>
+        </is>
+      </c>
+      <c r="C73" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="inlineStr">
+        <is>
+          <t>Silver Tribune</t>
+        </is>
+      </c>
+      <c r="E73" s="9" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="F73" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G73" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>CAT073</t>
+        </is>
+      </c>
+      <c r="B74" s="9" t="inlineStr">
+        <is>
+          <t>EVT019</t>
+        </is>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>SCVIP</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="inlineStr">
+        <is>
+          <t>Soundcheck VIP</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="F74" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="G74" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="inlineStr">
+        <is>
+          <t>CAT074</t>
+        </is>
+      </c>
+      <c r="B75" s="9" t="inlineStr">
+        <is>
+          <t>EVT019</t>
+        </is>
+      </c>
+      <c r="C75" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E75" s="9" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="F75" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G75" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="9" t="inlineStr">
+        <is>
+          <t>CAT075</t>
+        </is>
+      </c>
+      <c r="B76" s="9" t="inlineStr">
+        <is>
+          <t>EVT019</t>
+        </is>
+      </c>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="F76" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="G76" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="inlineStr">
+        <is>
+          <t>CAT076</t>
+        </is>
+      </c>
+      <c r="B77" s="9" t="inlineStr">
+        <is>
+          <t>EVT019</t>
+        </is>
+      </c>
+      <c r="C77" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>Gold Seat</t>
+        </is>
+      </c>
+      <c r="E77" s="9" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F77" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="G77" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="9" t="inlineStr">
+        <is>
+          <t>CAT077</t>
+        </is>
+      </c>
+      <c r="B78" s="9" t="inlineStr">
+        <is>
+          <t>EVT019</t>
+        </is>
+      </c>
+      <c r="C78" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>Silver Seat</t>
+        </is>
+      </c>
+      <c r="E78" s="9" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="F78" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G78" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="9" t="inlineStr">
+        <is>
+          <t>CAT078</t>
+        </is>
+      </c>
+      <c r="B79" s="9" t="inlineStr">
+        <is>
+          <t>EVT020</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E79" s="9" t="n">
+        <v>3900000</v>
+      </c>
+      <c r="F79" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="G79" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="9" t="inlineStr">
+        <is>
+          <t>CAT079</t>
+        </is>
+      </c>
+      <c r="B80" s="9" t="inlineStr">
+        <is>
+          <t>EVT020</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E80" s="9" t="n">
+        <v>2900000</v>
+      </c>
+      <c r="F80" s="9" t="n">
+        <v>95</v>
+      </c>
+      <c r="G80" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="inlineStr">
+        <is>
+          <t>CAT080</t>
+        </is>
+      </c>
+      <c r="B81" s="9" t="inlineStr">
+        <is>
+          <t>EVT020</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>Gold Lower</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="F81" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G81" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="9" t="inlineStr">
+        <is>
+          <t>CAT081</t>
+        </is>
+      </c>
+      <c r="B82" s="9" t="inlineStr">
+        <is>
+          <t>EVT020</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D82" s="9" t="inlineStr">
+        <is>
+          <t>Silver Upper</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="F82" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G82" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="inlineStr">
+        <is>
+          <t>CAT082</t>
+        </is>
+      </c>
+      <c r="B83" s="9" t="inlineStr">
+        <is>
+          <t>EVT021</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E83" s="9" t="n">
+        <v>5500000</v>
+      </c>
+      <c r="F83" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="G83" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="9" t="inlineStr">
+        <is>
+          <t>CAT083</t>
+        </is>
+      </c>
+      <c r="B84" s="9" t="inlineStr">
+        <is>
+          <t>EVT021</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D84" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E84" s="9" t="n">
+        <v>4200000</v>
+      </c>
+      <c r="F84" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="G84" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="9" t="inlineStr">
+        <is>
+          <t>CAT084</t>
+        </is>
+      </c>
+      <c r="B85" s="9" t="inlineStr">
+        <is>
+          <t>EVT021</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>Gold Lower</t>
+        </is>
+      </c>
+      <c r="E85" s="9" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="F85" s="9" t="n">
+        <v>160</v>
+      </c>
+      <c r="G85" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>CAT085</t>
+        </is>
+      </c>
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>EVT021</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D86" s="9" t="inlineStr">
+        <is>
+          <t>Silver Upper</t>
+        </is>
+      </c>
+      <c r="E86" s="9" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="F86" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="G86" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="9" t="inlineStr">
+        <is>
+          <t>CAT086</t>
+        </is>
+      </c>
+      <c r="B87" s="9" t="inlineStr">
+        <is>
+          <t>EVT022</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D87" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E87" s="9" t="n">
+        <v>4100000</v>
+      </c>
+      <c r="F87" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="G87" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>CAT087</t>
+        </is>
+      </c>
+      <c r="B88" s="9" t="inlineStr">
+        <is>
+          <t>EVT022</t>
+        </is>
+      </c>
+      <c r="C88" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D88" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E88" s="9" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="F88" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="G88" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="9" t="inlineStr">
+        <is>
+          <t>CAT088</t>
+        </is>
+      </c>
+      <c r="B89" s="9" t="inlineStr">
+        <is>
+          <t>EVT022</t>
+        </is>
+      </c>
+      <c r="C89" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D89" s="9" t="inlineStr">
+        <is>
+          <t>Gold Seat</t>
+        </is>
+      </c>
+      <c r="E89" s="9" t="n">
+        <v>2300000</v>
+      </c>
+      <c r="F89" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="G89" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>CAT089</t>
+        </is>
+      </c>
+      <c r="B90" s="9" t="inlineStr">
+        <is>
+          <t>EVT022</t>
+        </is>
+      </c>
+      <c r="C90" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D90" s="9" t="inlineStr">
+        <is>
+          <t>Silver Seat</t>
+        </is>
+      </c>
+      <c r="E90" s="9" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="F90" s="9" t="n">
+        <v>95</v>
+      </c>
+      <c r="G90" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="9" t="inlineStr">
+        <is>
+          <t>CAT090</t>
+        </is>
+      </c>
+      <c r="B91" s="9" t="inlineStr">
+        <is>
+          <t>EVT023</t>
+        </is>
+      </c>
+      <c r="C91" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D91" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E91" s="9" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="F91" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="G91" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>CAT091</t>
+        </is>
+      </c>
+      <c r="B92" s="9" t="inlineStr">
+        <is>
+          <t>EVT023</t>
+        </is>
+      </c>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D92" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E92" s="9" t="n">
+        <v>2700000</v>
+      </c>
+      <c r="F92" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G92" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="9" t="inlineStr">
+        <is>
+          <t>CAT092</t>
+        </is>
+      </c>
+      <c r="B93" s="9" t="inlineStr">
+        <is>
+          <t>EVT023</t>
+        </is>
+      </c>
+      <c r="C93" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D93" s="9" t="inlineStr">
+        <is>
+          <t>Gold Lower</t>
+        </is>
+      </c>
+      <c r="E93" s="9" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="F93" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="G93" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>CAT093</t>
+        </is>
+      </c>
+      <c r="B94" s="9" t="inlineStr">
+        <is>
+          <t>EVT023</t>
+        </is>
+      </c>
+      <c r="C94" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D94" s="9" t="inlineStr">
+        <is>
+          <t>Silver Upper</t>
+        </is>
+      </c>
+      <c r="E94" s="9" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="F94" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G94" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="9" t="inlineStr">
+        <is>
+          <t>CAT094</t>
+        </is>
+      </c>
+      <c r="B95" s="9" t="inlineStr">
+        <is>
+          <t>EVT024</t>
+        </is>
+      </c>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D95" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E95" s="9" t="n">
+        <v>3400000</v>
+      </c>
+      <c r="F95" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="G95" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>CAT095</t>
+        </is>
+      </c>
+      <c r="B96" s="9" t="inlineStr">
+        <is>
+          <t>EVT024</t>
+        </is>
+      </c>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D96" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E96" s="9" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F96" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G96" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="9" t="inlineStr">
+        <is>
+          <t>CAT096</t>
+        </is>
+      </c>
+      <c r="B97" s="9" t="inlineStr">
+        <is>
+          <t>EVT024</t>
+        </is>
+      </c>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D97" s="9" t="inlineStr">
+        <is>
+          <t>Gold Seat</t>
+        </is>
+      </c>
+      <c r="E97" s="9" t="n">
+        <v>1900000</v>
+      </c>
+      <c r="F97" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G97" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="9" t="inlineStr">
+        <is>
+          <t>CAT097</t>
+        </is>
+      </c>
+      <c r="B98" s="9" t="inlineStr">
+        <is>
+          <t>EVT024</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D98" s="9" t="inlineStr">
+        <is>
+          <t>Silver Seat</t>
+        </is>
+      </c>
+      <c r="E98" s="9" t="n">
+        <v>1350000</v>
+      </c>
+      <c r="F98" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="G98" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="9" t="inlineStr">
+        <is>
+          <t>CAT098</t>
+        </is>
+      </c>
+      <c r="B99" s="9" t="inlineStr">
+        <is>
+          <t>EVT025</t>
+        </is>
+      </c>
+      <c r="C99" s="9" t="inlineStr">
+        <is>
+          <t>SCVIP</t>
+        </is>
+      </c>
+      <c r="D99" s="9" t="inlineStr">
+        <is>
+          <t>Soundcheck VIP</t>
+        </is>
+      </c>
+      <c r="E99" s="9" t="n">
+        <v>4800000</v>
+      </c>
+      <c r="F99" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="G99" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="9" t="inlineStr">
+        <is>
+          <t>CAT099</t>
+        </is>
+      </c>
+      <c r="B100" s="9" t="inlineStr">
+        <is>
+          <t>EVT025</t>
+        </is>
+      </c>
+      <c r="C100" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D100" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E100" s="9" t="n">
+        <v>3900000</v>
+      </c>
+      <c r="F100" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G100" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="9" t="inlineStr">
+        <is>
+          <t>CAT100</t>
+        </is>
+      </c>
+      <c r="B101" s="9" t="inlineStr">
+        <is>
+          <t>EVT025</t>
+        </is>
+      </c>
+      <c r="C101" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D101" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E101" s="9" t="n">
+        <v>2900000</v>
+      </c>
+      <c r="F101" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="G101" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="9" t="inlineStr">
+        <is>
+          <t>CAT101</t>
+        </is>
+      </c>
+      <c r="B102" s="9" t="inlineStr">
+        <is>
+          <t>EVT025</t>
+        </is>
+      </c>
+      <c r="C102" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="inlineStr">
+        <is>
+          <t>Gold Lower</t>
+        </is>
+      </c>
+      <c r="E102" s="9" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="F102" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="G102" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="9" t="inlineStr">
+        <is>
+          <t>CAT102</t>
+        </is>
+      </c>
+      <c r="B103" s="9" t="inlineStr">
+        <is>
+          <t>EVT025</t>
+        </is>
+      </c>
+      <c r="C103" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D103" s="9" t="inlineStr">
+        <is>
+          <t>Silver Upper</t>
+        </is>
+      </c>
+      <c r="E103" s="9" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="F103" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G103" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="9" t="inlineStr">
+        <is>
+          <t>CAT103</t>
+        </is>
+      </c>
+      <c r="B104" s="9" t="inlineStr">
+        <is>
+          <t>EVT026</t>
+        </is>
+      </c>
+      <c r="C104" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D104" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E104" s="9" t="n">
+        <v>3700000</v>
+      </c>
+      <c r="F104" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="G104" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="9" t="inlineStr">
+        <is>
+          <t>CAT104</t>
+        </is>
+      </c>
+      <c r="B105" s="9" t="inlineStr">
+        <is>
+          <t>EVT026</t>
+        </is>
+      </c>
+      <c r="C105" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D105" s="9" t="inlineStr">
+        <is>
+          <t>A Reserved</t>
+        </is>
+      </c>
+      <c r="E105" s="9" t="n">
+        <v>2600000</v>
+      </c>
+      <c r="F105" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G105" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="9" t="inlineStr">
+        <is>
+          <t>CAT105</t>
+        </is>
+      </c>
+      <c r="B106" s="9" t="inlineStr">
+        <is>
+          <t>EVT026</t>
+        </is>
+      </c>
+      <c r="C106" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D106" s="9" t="inlineStr">
+        <is>
+          <t>B Reserved</t>
+        </is>
+      </c>
+      <c r="E106" s="9" t="n">
+        <v>1900000</v>
+      </c>
+      <c r="F106" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="G106" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="9" t="inlineStr">
+        <is>
+          <t>CAT106</t>
+        </is>
+      </c>
+      <c r="B107" s="9" t="inlineStr">
+        <is>
+          <t>EVT026</t>
+        </is>
+      </c>
+      <c r="C107" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D107" s="9" t="inlineStr">
+        <is>
+          <t>C Reserved</t>
+        </is>
+      </c>
+      <c r="E107" s="9" t="n">
+        <v>1400000</v>
+      </c>
+      <c r="F107" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G107" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="9" t="inlineStr">
+        <is>
+          <t>CAT107</t>
+        </is>
+      </c>
+      <c r="B108" s="9" t="inlineStr">
+        <is>
+          <t>EVT027</t>
+        </is>
+      </c>
+      <c r="C108" s="9" t="inlineStr">
+        <is>
+          <t>VVIP</t>
+        </is>
+      </c>
+      <c r="D108" s="9" t="inlineStr">
+        <is>
+          <t>VVIP Front</t>
+        </is>
+      </c>
+      <c r="E108" s="9" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="F108" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="G108" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="9" t="inlineStr">
+        <is>
+          <t>CAT108</t>
+        </is>
+      </c>
+      <c r="B109" s="9" t="inlineStr">
+        <is>
+          <t>EVT027</t>
+        </is>
+      </c>
+      <c r="C109" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D109" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E109" s="9" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="F109" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="G109" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="9" t="inlineStr">
+        <is>
+          <t>CAT109</t>
+        </is>
+      </c>
+      <c r="B110" s="9" t="inlineStr">
+        <is>
+          <t>EVT027</t>
+        </is>
+      </c>
+      <c r="C110" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>Zone A</t>
+        </is>
+      </c>
+      <c r="E110" s="9" t="n">
+        <v>2300000</v>
+      </c>
+      <c r="F110" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G110" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="9" t="inlineStr">
+        <is>
+          <t>CAT110</t>
+        </is>
+      </c>
+      <c r="B111" s="9" t="inlineStr">
+        <is>
+          <t>EVT027</t>
+        </is>
+      </c>
+      <c r="C111" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D111" s="9" t="inlineStr">
+        <is>
+          <t>Zone B</t>
+        </is>
+      </c>
+      <c r="E111" s="9" t="n">
+        <v>1650000</v>
+      </c>
+      <c r="F111" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="G111" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="9" t="inlineStr">
+        <is>
+          <t>CAT111</t>
+        </is>
+      </c>
+      <c r="B112" s="9" t="inlineStr">
+        <is>
+          <t>EVT028</t>
+        </is>
+      </c>
+      <c r="C112" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D112" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E112" s="9" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="F112" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="G112" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="9" t="inlineStr">
+        <is>
+          <t>CAT112</t>
+        </is>
+      </c>
+      <c r="B113" s="9" t="inlineStr">
+        <is>
+          <t>EVT028</t>
+        </is>
+      </c>
+      <c r="C113" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D113" s="9" t="inlineStr">
+        <is>
+          <t>Festival Standing</t>
+        </is>
+      </c>
+      <c r="E113" s="9" t="n">
+        <v>2300000</v>
+      </c>
+      <c r="F113" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="G113" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="9" t="inlineStr">
+        <is>
+          <t>CAT113</t>
+        </is>
+      </c>
+      <c r="B114" s="9" t="inlineStr">
+        <is>
+          <t>EVT028</t>
+        </is>
+      </c>
+      <c r="C114" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D114" s="9" t="inlineStr">
+        <is>
+          <t>Gold Tribune</t>
+        </is>
+      </c>
+      <c r="E114" s="9" t="n">
+        <v>1700000</v>
+      </c>
+      <c r="F114" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="G114" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="9" t="inlineStr">
+        <is>
+          <t>CAT114</t>
+        </is>
+      </c>
+      <c r="B115" s="9" t="inlineStr">
+        <is>
+          <t>EVT028</t>
+        </is>
+      </c>
+      <c r="C115" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="inlineStr">
+        <is>
+          <t>Silver Tribune</t>
+        </is>
+      </c>
+      <c r="E115" s="9" t="n">
+        <v>1150000</v>
+      </c>
+      <c r="F115" s="9" t="n">
+        <v>105</v>
+      </c>
+      <c r="G115" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="9" t="inlineStr">
+        <is>
+          <t>CAT115</t>
+        </is>
+      </c>
+      <c r="B116" s="9" t="inlineStr">
+        <is>
+          <t>EVT029</t>
+        </is>
+      </c>
+      <c r="C116" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D116" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E116" s="9" t="n">
+        <v>3300000</v>
+      </c>
+      <c r="F116" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="G116" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="9" t="inlineStr">
+        <is>
+          <t>CAT116</t>
+        </is>
+      </c>
+      <c r="B117" s="9" t="inlineStr">
+        <is>
+          <t>EVT029</t>
+        </is>
+      </c>
+      <c r="C117" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D117" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E117" s="9" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="F117" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G117" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="9" t="inlineStr">
+        <is>
+          <t>CAT117</t>
+        </is>
+      </c>
+      <c r="B118" s="9" t="inlineStr">
+        <is>
+          <t>EVT029</t>
+        </is>
+      </c>
+      <c r="C118" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D118" s="9" t="inlineStr">
+        <is>
+          <t>Gold Seat</t>
+        </is>
+      </c>
+      <c r="E118" s="9" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="F118" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G118" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="9" t="inlineStr">
+        <is>
+          <t>CAT118</t>
+        </is>
+      </c>
+      <c r="B119" s="9" t="inlineStr">
+        <is>
+          <t>EVT029</t>
+        </is>
+      </c>
+      <c r="C119" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D119" s="9" t="inlineStr">
+        <is>
+          <t>Silver Seat</t>
+        </is>
+      </c>
+      <c r="E119" s="9" t="n">
+        <v>1300000</v>
+      </c>
+      <c r="F119" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="G119" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="9" t="inlineStr">
+        <is>
+          <t>CAT119</t>
+        </is>
+      </c>
+      <c r="B120" s="9" t="inlineStr">
+        <is>
+          <t>EVT030</t>
+        </is>
+      </c>
+      <c r="C120" s="9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="D120" s="9" t="inlineStr">
+        <is>
+          <t>VIP Package</t>
+        </is>
+      </c>
+      <c r="E120" s="9" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="F120" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="G120" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="9" t="inlineStr">
+        <is>
+          <t>CAT120</t>
+        </is>
+      </c>
+      <c r="B121" s="9" t="inlineStr">
+        <is>
+          <t>EVT030</t>
+        </is>
+      </c>
+      <c r="C121" s="9" t="inlineStr">
+        <is>
+          <t>FLOOR</t>
+        </is>
+      </c>
+      <c r="D121" s="9" t="inlineStr">
+        <is>
+          <t>Floor Standing</t>
+        </is>
+      </c>
+      <c r="E121" s="9" t="n">
+        <v>3300000</v>
+      </c>
+      <c r="F121" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="G121" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="9" t="inlineStr">
+        <is>
+          <t>CAT121</t>
+        </is>
+      </c>
+      <c r="B122" s="9" t="inlineStr">
+        <is>
+          <t>EVT030</t>
+        </is>
+      </c>
+      <c r="C122" s="9" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D122" s="9" t="inlineStr">
+        <is>
+          <t>Gold Lower</t>
+        </is>
+      </c>
+      <c r="E122" s="9" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F122" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="G122" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="9" t="inlineStr">
+        <is>
+          <t>CAT122</t>
+        </is>
+      </c>
+      <c r="B123" s="9" t="inlineStr">
+        <is>
+          <t>EVT030</t>
+        </is>
+      </c>
+      <c r="C123" s="9" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="D123" s="9" t="inlineStr">
+        <is>
+          <t>Silver Upper</t>
+        </is>
+      </c>
+      <c r="E123" s="9" t="n">
+        <v>1750000</v>
+      </c>
+      <c r="F123" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G123" s="9" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>

</xml_diff>